<commit_message>
EM-16.1,16.2 - Rotina de edição de produtos
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5373D6B-09B7-430D-898D-9FA0F0EBE706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4569A6C3-4FB6-4E29-A385-C0C89C35EF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -646,7 +646,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -656,12 +656,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -678,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -734,13 +728,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1100,10 +1097,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="20">
+      <c r="A2" s="22">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1112,8 +1109,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="20"/>
-      <c r="B3" s="20"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1122,8 +1119,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1132,8 +1129,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1142,8 +1139,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1152,10 +1149,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="19">
+      <c r="A7" s="21">
         <v>2</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="21" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1166,8 +1163,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1179,8 +1176,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1190,10 +1187,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19">
+      <c r="A10" s="21">
         <v>3</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="21" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1204,8 +1201,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1214,8 +1211,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1224,8 +1221,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1235,8 +1232,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1245,8 +1242,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="16" t="s">
         <v>197</v>
       </c>
@@ -1255,10 +1252,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="19">
+      <c r="A16" s="21">
         <v>4</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="21" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1269,8 +1266,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
-      <c r="B17" s="19"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
       <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
@@ -1279,8 +1276,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
@@ -1289,8 +1286,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
@@ -1299,8 +1296,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
@@ -1309,8 +1306,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
-      <c r="B21" s="19"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
       <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
@@ -1319,8 +1316,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="19"/>
+      <c r="A22" s="21"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1329,10 +1326,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="19">
+      <c r="A23" s="21">
         <v>5</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="21" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1343,8 +1340,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="19"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1353,10 +1350,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19">
+      <c r="A25" s="21">
         <v>6</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="21" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1367,8 +1364,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
       <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1377,10 +1374,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="19">
+      <c r="A27" s="21">
         <v>7</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="21" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1391,8 +1388,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1457,10 +1454,10 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="19">
+      <c r="A33" s="21">
         <v>12</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="21" t="s">
         <v>48</v>
       </c>
       <c r="C33" s="17" t="s">
@@ -1471,8 +1468,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="19"/>
-      <c r="B34" s="19"/>
+      <c r="A34" s="21"/>
+      <c r="B34" s="21"/>
       <c r="C34" s="17" t="s">
         <v>134</v>
       </c>
@@ -1495,48 +1492,48 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="20">
+      <c r="A36" s="22">
         <v>14</v>
       </c>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="22" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="20"/>
-      <c r="B37" s="20"/>
+      <c r="A37" s="22"/>
+      <c r="B37" s="22"/>
       <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="20"/>
-      <c r="B38" s="20"/>
+      <c r="A38" s="22"/>
+      <c r="B38" s="22"/>
       <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="20"/>
-      <c r="B39" s="20"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="22"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="20"/>
-      <c r="B40" s="20"/>
+      <c r="A40" s="22"/>
+      <c r="B40" s="22"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="19">
+      <c r="A41" s="21">
         <v>15</v>
       </c>
-      <c r="B41" s="19" t="s">
+      <c r="B41" s="21" t="s">
         <v>55</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -1547,8 +1544,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="19"/>
-      <c r="B42" s="19"/>
+      <c r="A42" s="21"/>
+      <c r="B42" s="21"/>
       <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
@@ -1557,8 +1554,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="19"/>
-      <c r="B43" s="19"/>
+      <c r="A43" s="21"/>
+      <c r="B43" s="21"/>
       <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
@@ -1567,8 +1564,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="19"/>
-      <c r="B44" s="19"/>
+      <c r="A44" s="21"/>
+      <c r="B44" s="21"/>
       <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
@@ -1577,8 +1574,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="19"/>
-      <c r="B45" s="19"/>
+      <c r="A45" s="21"/>
+      <c r="B45" s="21"/>
       <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
@@ -1587,8 +1584,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
       <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
@@ -1597,42 +1594,42 @@
       </c>
     </row>
     <row r="47" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="19">
+      <c r="A47" s="21">
         <v>16</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="C47" s="21" t="s">
+      <c r="C47" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="19" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="19"/>
-      <c r="B48" s="19"/>
-      <c r="C48" s="1" t="s">
+      <c r="A48" s="21"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D48" s="20" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="19"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="1" t="s">
+      <c r="A49" s="21"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D49" s="20" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="19"/>
-      <c r="B50" s="19"/>
+      <c r="A50" s="21"/>
+      <c r="B50" s="21"/>
       <c r="C50" s="1" t="s">
         <v>64</v>
       </c>
@@ -1641,8 +1638,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="19"/>
-      <c r="B51" s="19"/>
+      <c r="A51" s="21"/>
+      <c r="B51" s="21"/>
       <c r="C51" s="1" t="s">
         <v>65</v>
       </c>
@@ -1651,8 +1648,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="19"/>
-      <c r="B52" s="19"/>
+      <c r="A52" s="21"/>
+      <c r="B52" s="21"/>
       <c r="C52" s="1" t="s">
         <v>68</v>
       </c>
@@ -1661,8 +1658,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="19"/>
-      <c r="B53" s="19"/>
+      <c r="A53" s="21"/>
+      <c r="B53" s="21"/>
       <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
@@ -1671,8 +1668,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="19"/>
-      <c r="B54" s="19"/>
+      <c r="A54" s="21"/>
+      <c r="B54" s="21"/>
       <c r="C54" s="1" t="s">
         <v>74</v>
       </c>
@@ -1681,8 +1678,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="19"/>
-      <c r="B55" s="19"/>
+      <c r="A55" s="21"/>
+      <c r="B55" s="21"/>
       <c r="C55" s="1" t="s">
         <v>75</v>
       </c>
@@ -1691,8 +1688,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="19"/>
-      <c r="B56" s="19"/>
+      <c r="A56" s="21"/>
+      <c r="B56" s="21"/>
       <c r="C56" s="1" t="s">
         <v>76</v>
       </c>
@@ -1701,10 +1698,10 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="19">
+      <c r="A57" s="21">
         <v>17</v>
       </c>
-      <c r="B57" s="19" t="s">
+      <c r="B57" s="21" t="s">
         <v>77</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -1715,8 +1712,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="19"/>
-      <c r="B58" s="19"/>
+      <c r="A58" s="21"/>
+      <c r="B58" s="21"/>
       <c r="C58" s="1" t="s">
         <v>79</v>
       </c>
@@ -1725,8 +1722,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="19"/>
-      <c r="B59" s="19"/>
+      <c r="A59" s="21"/>
+      <c r="B59" s="21"/>
       <c r="C59" s="1" t="s">
         <v>80</v>
       </c>
@@ -1735,8 +1732,8 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="19"/>
-      <c r="B60" s="19"/>
+      <c r="A60" s="21"/>
+      <c r="B60" s="21"/>
       <c r="C60" s="1" t="s">
         <v>81</v>
       </c>
@@ -1745,10 +1742,10 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="19">
+      <c r="A61" s="21">
         <v>18</v>
       </c>
-      <c r="B61" s="19" t="s">
+      <c r="B61" s="21" t="s">
         <v>82</v>
       </c>
       <c r="C61" s="1" t="s">
@@ -1759,8 +1756,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="19"/>
-      <c r="B62" s="19"/>
+      <c r="A62" s="21"/>
+      <c r="B62" s="21"/>
       <c r="C62" s="1" t="s">
         <v>84</v>
       </c>
@@ -1769,8 +1766,8 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="19"/>
-      <c r="B63" s="19"/>
+      <c r="A63" s="21"/>
+      <c r="B63" s="21"/>
       <c r="C63" s="1" t="s">
         <v>85</v>
       </c>
@@ -1779,8 +1776,8 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="19"/>
-      <c r="B64" s="19"/>
+      <c r="A64" s="21"/>
+      <c r="B64" s="21"/>
       <c r="C64" s="1" t="s">
         <v>86</v>
       </c>
@@ -1789,10 +1786,10 @@
       </c>
     </row>
     <row r="65" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="19">
+      <c r="A65" s="21">
         <v>19</v>
       </c>
-      <c r="B65" s="19" t="s">
+      <c r="B65" s="21" t="s">
         <v>87</v>
       </c>
       <c r="C65" s="1" t="s">
@@ -1803,8 +1800,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="19"/>
-      <c r="B66" s="19"/>
+      <c r="A66" s="21"/>
+      <c r="B66" s="21"/>
       <c r="C66" s="1" t="s">
         <v>89</v>
       </c>
@@ -1813,8 +1810,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="19"/>
-      <c r="B67" s="19"/>
+      <c r="A67" s="21"/>
+      <c r="B67" s="21"/>
       <c r="C67" s="1" t="s">
         <v>90</v>
       </c>
@@ -1823,8 +1820,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="19"/>
-      <c r="B68" s="19"/>
+      <c r="A68" s="21"/>
+      <c r="B68" s="21"/>
       <c r="C68" s="1" t="s">
         <v>91</v>
       </c>
@@ -1833,10 +1830,10 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="19">
+      <c r="A69" s="21">
         <v>20</v>
       </c>
-      <c r="B69" s="19" t="s">
+      <c r="B69" s="21" t="s">
         <v>92</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -1847,8 +1844,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="19"/>
-      <c r="B70" s="19"/>
+      <c r="A70" s="21"/>
+      <c r="B70" s="21"/>
       <c r="C70" s="1" t="s">
         <v>94</v>
       </c>
@@ -1857,8 +1854,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="19"/>
-      <c r="B71" s="19"/>
+      <c r="A71" s="21"/>
+      <c r="B71" s="21"/>
       <c r="C71" s="1" t="s">
         <v>95</v>
       </c>
@@ -1867,8 +1864,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="19"/>
-      <c r="B72" s="19"/>
+      <c r="A72" s="21"/>
+      <c r="B72" s="21"/>
       <c r="C72" s="1" t="s">
         <v>96</v>
       </c>
@@ -1877,10 +1874,10 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="19">
+      <c r="A73" s="21">
         <v>21</v>
       </c>
-      <c r="B73" s="19" t="s">
+      <c r="B73" s="21" t="s">
         <v>97</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -1891,8 +1888,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="19"/>
-      <c r="B74" s="19"/>
+      <c r="A74" s="21"/>
+      <c r="B74" s="21"/>
       <c r="C74" s="1" t="s">
         <v>99</v>
       </c>
@@ -1901,8 +1898,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="19"/>
-      <c r="B75" s="19"/>
+      <c r="A75" s="21"/>
+      <c r="B75" s="21"/>
       <c r="C75" s="1" t="s">
         <v>100</v>
       </c>
@@ -1911,8 +1908,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="19"/>
-      <c r="B76" s="19"/>
+      <c r="A76" s="21"/>
+      <c r="B76" s="21"/>
       <c r="C76" s="1" t="s">
         <v>101</v>
       </c>
@@ -1921,10 +1918,10 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="19">
+      <c r="A77" s="21">
         <v>22</v>
       </c>
-      <c r="B77" s="19" t="s">
+      <c r="B77" s="21" t="s">
         <v>102</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -1935,8 +1932,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="19"/>
-      <c r="B78" s="19"/>
+      <c r="A78" s="21"/>
+      <c r="B78" s="21"/>
       <c r="C78" s="1" t="s">
         <v>104</v>
       </c>
@@ -1945,8 +1942,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="19"/>
-      <c r="B79" s="19"/>
+      <c r="A79" s="21"/>
+      <c r="B79" s="21"/>
       <c r="C79" s="1" t="s">
         <v>105</v>
       </c>
@@ -1955,8 +1952,8 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="19"/>
-      <c r="B80" s="19"/>
+      <c r="A80" s="21"/>
+      <c r="B80" s="21"/>
       <c r="C80" s="1" t="s">
         <v>106</v>
       </c>
@@ -1965,8 +1962,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="19"/>
-      <c r="B81" s="19"/>
+      <c r="A81" s="21"/>
+      <c r="B81" s="21"/>
       <c r="C81" s="1" t="s">
         <v>107</v>
       </c>
@@ -1975,10 +1972,10 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="19">
+      <c r="A82" s="21">
         <v>23</v>
       </c>
-      <c r="B82" s="19" t="s">
+      <c r="B82" s="21" t="s">
         <v>108</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -1989,8 +1986,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="19"/>
-      <c r="B83" s="19"/>
+      <c r="A83" s="21"/>
+      <c r="B83" s="21"/>
       <c r="C83" s="1" t="s">
         <v>110</v>
       </c>
@@ -1999,8 +1996,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="19"/>
-      <c r="B84" s="19"/>
+      <c r="A84" s="21"/>
+      <c r="B84" s="21"/>
       <c r="C84" s="1" t="s">
         <v>111</v>
       </c>
@@ -2009,10 +2006,10 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="19">
+      <c r="A85" s="21">
         <v>24</v>
       </c>
-      <c r="B85" s="19" t="s">
+      <c r="B85" s="21" t="s">
         <v>112</v>
       </c>
       <c r="C85" s="1" t="s">
@@ -2023,8 +2020,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="19"/>
-      <c r="B86" s="19"/>
+      <c r="A86" s="21"/>
+      <c r="B86" s="21"/>
       <c r="C86" s="1" t="s">
         <v>114</v>
       </c>
@@ -2033,8 +2030,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="19"/>
-      <c r="B87" s="19"/>
+      <c r="A87" s="21"/>
+      <c r="B87" s="21"/>
       <c r="C87" s="1" t="s">
         <v>115</v>
       </c>
@@ -2043,10 +2040,10 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="19">
+      <c r="A88" s="21">
         <v>25</v>
       </c>
-      <c r="B88" s="19" t="s">
+      <c r="B88" s="21" t="s">
         <v>116</v>
       </c>
       <c r="C88" s="1" t="s">
@@ -2057,8 +2054,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="19"/>
-      <c r="B89" s="19"/>
+      <c r="A89" s="21"/>
+      <c r="B89" s="21"/>
       <c r="C89" s="1" t="s">
         <v>118</v>
       </c>
@@ -2067,8 +2064,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="19"/>
-      <c r="B90" s="19"/>
+      <c r="A90" s="21"/>
+      <c r="B90" s="21"/>
       <c r="C90" s="1" t="s">
         <v>119</v>
       </c>
@@ -2077,8 +2074,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="19"/>
-      <c r="B91" s="19"/>
+      <c r="A91" s="21"/>
+      <c r="B91" s="21"/>
       <c r="C91" s="1" t="s">
         <v>120</v>
       </c>

</xml_diff>

<commit_message>
EM-16.8 - Baixa de estoque + validação se tem estoque disponivel na compra
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4569A6C3-4FB6-4E29-A385-C0C89C35EF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D6AB38-18DC-44B8-BCAB-3F903D2291EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>US</t>
   </si>
@@ -625,6 +625,9 @@
   </si>
   <si>
     <t>16.10</t>
+  </si>
+  <si>
+    <t>Feito na 16.2</t>
   </si>
 </sst>
 </file>
@@ -646,7 +649,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -656,6 +659,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -672,7 +687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -738,6 +753,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1617,7 +1638,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="21"/>
       <c r="B49" s="21"/>
       <c r="C49" s="20" t="s">
@@ -1627,7 +1648,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="21"/>
       <c r="B50" s="21"/>
       <c r="C50" s="1" t="s">
@@ -1637,27 +1658,30 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="21"/>
       <c r="B51" s="21"/>
-      <c r="C51" s="1" t="s">
+      <c r="C51" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D51" s="7" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="21"/>
       <c r="B52" s="21"/>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D52" s="24" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="21"/>
       <c r="B53" s="21"/>
       <c r="C53" s="1" t="s">
@@ -1667,7 +1691,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="21"/>
       <c r="B54" s="21"/>
       <c r="C54" s="1" t="s">
@@ -1677,17 +1701,17 @@
         <v>149</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="21"/>
       <c r="B55" s="21"/>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="D55" s="23" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="21"/>
       <c r="B56" s="21"/>
       <c r="C56" s="1" t="s">
@@ -1697,7 +1721,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="21">
         <v>17</v>
       </c>
@@ -1711,7 +1735,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="21"/>
       <c r="B58" s="21"/>
       <c r="C58" s="1" t="s">
@@ -1721,7 +1745,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="21"/>
       <c r="B59" s="21"/>
       <c r="C59" s="1" t="s">
@@ -1731,7 +1755,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="21"/>
       <c r="B60" s="21"/>
       <c r="C60" s="1" t="s">
@@ -1741,7 +1765,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="21">
         <v>18</v>
       </c>
@@ -1755,7 +1779,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="21"/>
       <c r="B62" s="21"/>
       <c r="C62" s="1" t="s">
@@ -1765,7 +1789,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="21"/>
       <c r="B63" s="21"/>
       <c r="C63" s="1" t="s">
@@ -1775,7 +1799,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="21"/>
       <c r="B64" s="21"/>
       <c r="C64" s="1" t="s">

</xml_diff>

<commit_message>
EM-18.1 - Tabela de avaliações de produtos
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D6AB38-18DC-44B8-BCAB-3F903D2291EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5A1413-2A35-4415-B028-72E5EA8CAD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -649,7 +649,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -659,12 +659,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -749,16 +743,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1118,10 +1112,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22">
+      <c r="A2" s="23">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1130,8 +1124,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="22"/>
-      <c r="B3" s="22"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="23"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1140,8 +1134,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1150,8 +1144,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1160,8 +1154,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="23"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1170,10 +1164,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="21">
+      <c r="A7" s="24">
         <v>2</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="24" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1184,8 +1178,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1197,8 +1191,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1208,10 +1202,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21">
+      <c r="A10" s="24">
         <v>3</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="24" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1222,8 +1216,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1232,8 +1226,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1242,8 +1236,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1253,8 +1247,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1263,8 +1257,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="16" t="s">
         <v>197</v>
       </c>
@@ -1273,10 +1267,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="21">
+      <c r="A16" s="24">
         <v>4</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="24" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1287,8 +1281,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
       <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
@@ -1297,8 +1291,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
       <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
@@ -1307,8 +1301,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
@@ -1317,8 +1311,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
@@ -1327,8 +1321,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
@@ -1337,8 +1331,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1347,10 +1341,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="21">
+      <c r="A23" s="24">
         <v>5</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="24" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1361,8 +1355,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1371,10 +1365,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="21">
+      <c r="A25" s="24">
         <v>6</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="24" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1385,8 +1379,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
       <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1395,10 +1389,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="21">
+      <c r="A27" s="24">
         <v>7</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="24" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1409,8 +1403,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1475,10 +1469,10 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="21">
+      <c r="A33" s="24">
         <v>12</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="24" t="s">
         <v>48</v>
       </c>
       <c r="C33" s="17" t="s">
@@ -1489,8 +1483,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
       <c r="C34" s="17" t="s">
         <v>134</v>
       </c>
@@ -1513,48 +1507,48 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="22">
+      <c r="A36" s="23">
         <v>14</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="23" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22"/>
+      <c r="A37" s="23"/>
+      <c r="B37" s="23"/>
       <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="22"/>
-      <c r="B38" s="22"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
       <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="21">
+      <c r="A41" s="24">
         <v>15</v>
       </c>
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="24" t="s">
         <v>55</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -1565,8 +1559,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="21"/>
-      <c r="B42" s="21"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
       <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
@@ -1575,8 +1569,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="21"/>
-      <c r="B43" s="21"/>
+      <c r="A43" s="24"/>
+      <c r="B43" s="24"/>
       <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
@@ -1585,8 +1579,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="21"/>
-      <c r="B44" s="21"/>
+      <c r="A44" s="24"/>
+      <c r="B44" s="24"/>
       <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
@@ -1595,8 +1589,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="21"/>
-      <c r="B45" s="21"/>
+      <c r="A45" s="24"/>
+      <c r="B45" s="24"/>
       <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
@@ -1605,8 +1599,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="21"/>
-      <c r="B46" s="21"/>
+      <c r="A46" s="24"/>
+      <c r="B46" s="24"/>
       <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
@@ -1615,10 +1609,10 @@
       </c>
     </row>
     <row r="47" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="21">
+      <c r="A47" s="24">
         <v>16</v>
       </c>
-      <c r="B47" s="21" t="s">
+      <c r="B47" s="24" t="s">
         <v>73</v>
       </c>
       <c r="C47" s="19" t="s">
@@ -1629,8 +1623,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="21"/>
-      <c r="B48" s="21"/>
+      <c r="A48" s="24"/>
+      <c r="B48" s="24"/>
       <c r="C48" s="20" t="s">
         <v>62</v>
       </c>
@@ -1639,8 +1633,8 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="21"/>
-      <c r="B49" s="21"/>
+      <c r="A49" s="24"/>
+      <c r="B49" s="24"/>
       <c r="C49" s="20" t="s">
         <v>63</v>
       </c>
@@ -1649,8 +1643,8 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="21"/>
-      <c r="B50" s="21"/>
+      <c r="A50" s="24"/>
+      <c r="B50" s="24"/>
       <c r="C50" s="1" t="s">
         <v>64</v>
       </c>
@@ -1659,8 +1653,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="21"/>
-      <c r="B51" s="21"/>
+      <c r="A51" s="24"/>
+      <c r="B51" s="24"/>
       <c r="C51" s="7" t="s">
         <v>65</v>
       </c>
@@ -1669,12 +1663,12 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="21"/>
-      <c r="B52" s="21"/>
-      <c r="C52" s="24" t="s">
+      <c r="A52" s="24"/>
+      <c r="B52" s="24"/>
+      <c r="C52" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D52" s="24" t="s">
+      <c r="D52" s="22" t="s">
         <v>147</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -1682,8 +1676,8 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="21"/>
-      <c r="B53" s="21"/>
+      <c r="A53" s="24"/>
+      <c r="B53" s="24"/>
       <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
@@ -1692,8 +1686,8 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="21"/>
-      <c r="B54" s="21"/>
+      <c r="A54" s="24"/>
+      <c r="B54" s="24"/>
       <c r="C54" s="1" t="s">
         <v>74</v>
       </c>
@@ -1702,18 +1696,18 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="21"/>
-      <c r="B55" s="21"/>
-      <c r="C55" s="23" t="s">
+      <c r="A55" s="24"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="D55" s="23" t="s">
+      <c r="D55" s="21" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="21"/>
-      <c r="B56" s="21"/>
+      <c r="A56" s="24"/>
+      <c r="B56" s="24"/>
       <c r="C56" s="1" t="s">
         <v>76</v>
       </c>
@@ -1722,10 +1716,10 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="21">
+      <c r="A57" s="24">
         <v>17</v>
       </c>
-      <c r="B57" s="21" t="s">
+      <c r="B57" s="24" t="s">
         <v>77</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -1736,8 +1730,8 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="21"/>
-      <c r="B58" s="21"/>
+      <c r="A58" s="24"/>
+      <c r="B58" s="24"/>
       <c r="C58" s="1" t="s">
         <v>79</v>
       </c>
@@ -1746,8 +1740,8 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="21"/>
-      <c r="B59" s="21"/>
+      <c r="A59" s="24"/>
+      <c r="B59" s="24"/>
       <c r="C59" s="1" t="s">
         <v>80</v>
       </c>
@@ -1756,8 +1750,8 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="21"/>
-      <c r="B60" s="21"/>
+      <c r="A60" s="24"/>
+      <c r="B60" s="24"/>
       <c r="C60" s="1" t="s">
         <v>81</v>
       </c>
@@ -1766,22 +1760,22 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="21">
+      <c r="A61" s="24">
         <v>18</v>
       </c>
-      <c r="B61" s="21" t="s">
+      <c r="B61" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="D61" s="21" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="21"/>
-      <c r="B62" s="21"/>
+      <c r="A62" s="24"/>
+      <c r="B62" s="24"/>
       <c r="C62" s="1" t="s">
         <v>84</v>
       </c>
@@ -1790,8 +1784,8 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="21"/>
-      <c r="B63" s="21"/>
+      <c r="A63" s="24"/>
+      <c r="B63" s="24"/>
       <c r="C63" s="1" t="s">
         <v>85</v>
       </c>
@@ -1800,8 +1794,8 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="21"/>
-      <c r="B64" s="21"/>
+      <c r="A64" s="24"/>
+      <c r="B64" s="24"/>
       <c r="C64" s="1" t="s">
         <v>86</v>
       </c>
@@ -1810,10 +1804,10 @@
       </c>
     </row>
     <row r="65" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="21">
+      <c r="A65" s="24">
         <v>19</v>
       </c>
-      <c r="B65" s="21" t="s">
+      <c r="B65" s="24" t="s">
         <v>87</v>
       </c>
       <c r="C65" s="1" t="s">
@@ -1824,8 +1818,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="21"/>
-      <c r="B66" s="21"/>
+      <c r="A66" s="24"/>
+      <c r="B66" s="24"/>
       <c r="C66" s="1" t="s">
         <v>89</v>
       </c>
@@ -1834,8 +1828,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="21"/>
-      <c r="B67" s="21"/>
+      <c r="A67" s="24"/>
+      <c r="B67" s="24"/>
       <c r="C67" s="1" t="s">
         <v>90</v>
       </c>
@@ -1844,8 +1838,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="21"/>
-      <c r="B68" s="21"/>
+      <c r="A68" s="24"/>
+      <c r="B68" s="24"/>
       <c r="C68" s="1" t="s">
         <v>91</v>
       </c>
@@ -1854,10 +1848,10 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="21">
+      <c r="A69" s="24">
         <v>20</v>
       </c>
-      <c r="B69" s="21" t="s">
+      <c r="B69" s="24" t="s">
         <v>92</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -1868,8 +1862,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="21"/>
-      <c r="B70" s="21"/>
+      <c r="A70" s="24"/>
+      <c r="B70" s="24"/>
       <c r="C70" s="1" t="s">
         <v>94</v>
       </c>
@@ -1878,8 +1872,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="21"/>
-      <c r="B71" s="21"/>
+      <c r="A71" s="24"/>
+      <c r="B71" s="24"/>
       <c r="C71" s="1" t="s">
         <v>95</v>
       </c>
@@ -1888,8 +1882,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="21"/>
-      <c r="B72" s="21"/>
+      <c r="A72" s="24"/>
+      <c r="B72" s="24"/>
       <c r="C72" s="1" t="s">
         <v>96</v>
       </c>
@@ -1898,10 +1892,10 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="21">
+      <c r="A73" s="24">
         <v>21</v>
       </c>
-      <c r="B73" s="21" t="s">
+      <c r="B73" s="24" t="s">
         <v>97</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -1912,8 +1906,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="21"/>
-      <c r="B74" s="21"/>
+      <c r="A74" s="24"/>
+      <c r="B74" s="24"/>
       <c r="C74" s="1" t="s">
         <v>99</v>
       </c>
@@ -1922,8 +1916,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="21"/>
-      <c r="B75" s="21"/>
+      <c r="A75" s="24"/>
+      <c r="B75" s="24"/>
       <c r="C75" s="1" t="s">
         <v>100</v>
       </c>
@@ -1932,8 +1926,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="21"/>
-      <c r="B76" s="21"/>
+      <c r="A76" s="24"/>
+      <c r="B76" s="24"/>
       <c r="C76" s="1" t="s">
         <v>101</v>
       </c>
@@ -1942,10 +1936,10 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="21">
+      <c r="A77" s="24">
         <v>22</v>
       </c>
-      <c r="B77" s="21" t="s">
+      <c r="B77" s="24" t="s">
         <v>102</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -1956,8 +1950,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="21"/>
-      <c r="B78" s="21"/>
+      <c r="A78" s="24"/>
+      <c r="B78" s="24"/>
       <c r="C78" s="1" t="s">
         <v>104</v>
       </c>
@@ -1966,8 +1960,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="21"/>
-      <c r="B79" s="21"/>
+      <c r="A79" s="24"/>
+      <c r="B79" s="24"/>
       <c r="C79" s="1" t="s">
         <v>105</v>
       </c>
@@ -1976,8 +1970,8 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="21"/>
-      <c r="B80" s="21"/>
+      <c r="A80" s="24"/>
+      <c r="B80" s="24"/>
       <c r="C80" s="1" t="s">
         <v>106</v>
       </c>
@@ -1986,8 +1980,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="21"/>
-      <c r="B81" s="21"/>
+      <c r="A81" s="24"/>
+      <c r="B81" s="24"/>
       <c r="C81" s="1" t="s">
         <v>107</v>
       </c>
@@ -1996,10 +1990,10 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="21">
+      <c r="A82" s="24">
         <v>23</v>
       </c>
-      <c r="B82" s="21" t="s">
+      <c r="B82" s="24" t="s">
         <v>108</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -2010,8 +2004,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="21"/>
-      <c r="B83" s="21"/>
+      <c r="A83" s="24"/>
+      <c r="B83" s="24"/>
       <c r="C83" s="1" t="s">
         <v>110</v>
       </c>
@@ -2020,8 +2014,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="21"/>
-      <c r="B84" s="21"/>
+      <c r="A84" s="24"/>
+      <c r="B84" s="24"/>
       <c r="C84" s="1" t="s">
         <v>111</v>
       </c>
@@ -2030,10 +2024,10 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="21">
+      <c r="A85" s="24">
         <v>24</v>
       </c>
-      <c r="B85" s="21" t="s">
+      <c r="B85" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C85" s="1" t="s">
@@ -2044,8 +2038,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="21"/>
-      <c r="B86" s="21"/>
+      <c r="A86" s="24"/>
+      <c r="B86" s="24"/>
       <c r="C86" s="1" t="s">
         <v>114</v>
       </c>
@@ -2054,8 +2048,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="21"/>
-      <c r="B87" s="21"/>
+      <c r="A87" s="24"/>
+      <c r="B87" s="24"/>
       <c r="C87" s="1" t="s">
         <v>115</v>
       </c>
@@ -2064,10 +2058,10 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="21">
+      <c r="A88" s="24">
         <v>25</v>
       </c>
-      <c r="B88" s="21" t="s">
+      <c r="B88" s="24" t="s">
         <v>116</v>
       </c>
       <c r="C88" s="1" t="s">
@@ -2078,8 +2072,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="21"/>
-      <c r="B89" s="21"/>
+      <c r="A89" s="24"/>
+      <c r="B89" s="24"/>
       <c r="C89" s="1" t="s">
         <v>118</v>
       </c>
@@ -2088,8 +2082,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="21"/>
-      <c r="B90" s="21"/>
+      <c r="A90" s="24"/>
+      <c r="B90" s="24"/>
       <c r="C90" s="1" t="s">
         <v>119</v>
       </c>
@@ -2098,8 +2092,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="21"/>
-      <c r="B91" s="21"/>
+      <c r="A91" s="24"/>
+      <c r="B91" s="24"/>
       <c r="C91" s="1" t="s">
         <v>120</v>
       </c>
@@ -2109,14 +2103,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A16:A22"/>
-    <mergeCell ref="B16:B22"/>
-    <mergeCell ref="A10:A15"/>
-    <mergeCell ref="B10:B15"/>
+    <mergeCell ref="B85:B87"/>
+    <mergeCell ref="B88:B91"/>
+    <mergeCell ref="A85:A87"/>
+    <mergeCell ref="A88:A91"/>
+    <mergeCell ref="B73:B76"/>
+    <mergeCell ref="A73:A76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="A77:A81"/>
+    <mergeCell ref="A82:A84"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="B61:B64"/>
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="B65:B68"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B57:B60"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="B41:B46"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B47:B56"/>
+    <mergeCell ref="A47:A56"/>
     <mergeCell ref="B36:B40"/>
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="B7:B9"/>
@@ -2127,28 +2135,14 @@
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B57:B60"/>
-    <mergeCell ref="A57:A60"/>
-    <mergeCell ref="B41:B46"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B47:B56"/>
-    <mergeCell ref="A47:A56"/>
-    <mergeCell ref="B61:B64"/>
-    <mergeCell ref="A61:A64"/>
-    <mergeCell ref="B65:B68"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="B69:B72"/>
-    <mergeCell ref="A69:A72"/>
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="B88:B91"/>
-    <mergeCell ref="A85:A87"/>
-    <mergeCell ref="A88:A91"/>
-    <mergeCell ref="B73:B76"/>
-    <mergeCell ref="A73:A76"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="A77:A81"/>
-    <mergeCell ref="A82:A84"/>
-    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="B10:B15"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
EM-18.2 - Tela para avaliação de produtos comprados
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5A1413-2A35-4415-B028-72E5EA8CAD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FFF83C-B2CE-4D42-A186-0AE67DD3ADEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -649,7 +649,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -659,6 +659,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -681,7 +687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -747,6 +753,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1112,10 +1121,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="23">
+      <c r="A2" s="24">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1124,8 +1133,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="24"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1134,8 +1143,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1144,8 +1153,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1154,8 +1163,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1164,10 +1173,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="24">
+      <c r="A7" s="25">
         <v>2</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="25" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1178,8 +1187,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1191,8 +1200,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1202,10 +1211,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="24">
+      <c r="A10" s="25">
         <v>3</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="25" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1216,8 +1225,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1226,8 +1235,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1236,8 +1245,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="25"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1247,8 +1256,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="24"/>
-      <c r="B14" s="24"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="25"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1257,8 +1266,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
       <c r="C15" s="16" t="s">
         <v>197</v>
       </c>
@@ -1267,10 +1276,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="24">
+      <c r="A16" s="25">
         <v>4</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="25" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1281,8 +1290,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="24"/>
-      <c r="B17" s="24"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
       <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
@@ -1291,8 +1300,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="25"/>
       <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
@@ -1301,8 +1310,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="25"/>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
@@ -1311,8 +1320,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="25"/>
       <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
@@ -1321,8 +1330,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
       <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
@@ -1331,8 +1340,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="24"/>
-      <c r="B22" s="24"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1341,10 +1350,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="24">
+      <c r="A23" s="25">
         <v>5</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="25" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1355,8 +1364,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="24"/>
-      <c r="B24" s="24"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="25"/>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1365,10 +1374,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="24">
+      <c r="A25" s="25">
         <v>6</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1379,8 +1388,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="24"/>
-      <c r="B26" s="24"/>
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
       <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1389,10 +1398,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="24">
+      <c r="A27" s="25">
         <v>7</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1403,8 +1412,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="24"/>
-      <c r="B28" s="24"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1469,10 +1478,10 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="24">
+      <c r="A33" s="25">
         <v>12</v>
       </c>
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="25" t="s">
         <v>48</v>
       </c>
       <c r="C33" s="17" t="s">
@@ -1483,8 +1492,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="24"/>
-      <c r="B34" s="24"/>
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
       <c r="C34" s="17" t="s">
         <v>134</v>
       </c>
@@ -1507,48 +1516,48 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="23">
+      <c r="A36" s="24">
         <v>14</v>
       </c>
-      <c r="B36" s="23" t="s">
+      <c r="B36" s="24" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="23"/>
-      <c r="B37" s="23"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
       <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="23"/>
-      <c r="B38" s="23"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="24"/>
       <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="23"/>
-      <c r="B39" s="23"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="23"/>
-      <c r="B40" s="23"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="24">
+      <c r="A41" s="25">
         <v>15</v>
       </c>
-      <c r="B41" s="24" t="s">
+      <c r="B41" s="25" t="s">
         <v>55</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -1559,8 +1568,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="24"/>
-      <c r="B42" s="24"/>
+      <c r="A42" s="25"/>
+      <c r="B42" s="25"/>
       <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
@@ -1569,8 +1578,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="24"/>
-      <c r="B43" s="24"/>
+      <c r="A43" s="25"/>
+      <c r="B43" s="25"/>
       <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
@@ -1579,8 +1588,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="24"/>
-      <c r="B44" s="24"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="25"/>
       <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
@@ -1589,8 +1598,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="24"/>
-      <c r="B45" s="24"/>
+      <c r="A45" s="25"/>
+      <c r="B45" s="25"/>
       <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
@@ -1599,8 +1608,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="24"/>
-      <c r="B46" s="24"/>
+      <c r="A46" s="25"/>
+      <c r="B46" s="25"/>
       <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
@@ -1609,10 +1618,10 @@
       </c>
     </row>
     <row r="47" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="24">
+      <c r="A47" s="25">
         <v>16</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="25" t="s">
         <v>73</v>
       </c>
       <c r="C47" s="19" t="s">
@@ -1623,8 +1632,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="24"/>
-      <c r="B48" s="24"/>
+      <c r="A48" s="25"/>
+      <c r="B48" s="25"/>
       <c r="C48" s="20" t="s">
         <v>62</v>
       </c>
@@ -1633,8 +1642,8 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="24"/>
-      <c r="B49" s="24"/>
+      <c r="A49" s="25"/>
+      <c r="B49" s="25"/>
       <c r="C49" s="20" t="s">
         <v>63</v>
       </c>
@@ -1643,8 +1652,8 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="24"/>
-      <c r="B50" s="24"/>
+      <c r="A50" s="25"/>
+      <c r="B50" s="25"/>
       <c r="C50" s="1" t="s">
         <v>64</v>
       </c>
@@ -1653,8 +1662,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="24"/>
-      <c r="B51" s="24"/>
+      <c r="A51" s="25"/>
+      <c r="B51" s="25"/>
       <c r="C51" s="7" t="s">
         <v>65</v>
       </c>
@@ -1663,12 +1672,12 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="24"/>
-      <c r="B52" s="24"/>
-      <c r="C52" s="22" t="s">
+      <c r="A52" s="25"/>
+      <c r="B52" s="25"/>
+      <c r="C52" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D52" s="22" t="s">
+      <c r="D52" s="23" t="s">
         <v>147</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -1676,8 +1685,8 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="24"/>
-      <c r="B53" s="24"/>
+      <c r="A53" s="25"/>
+      <c r="B53" s="25"/>
       <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
@@ -1686,8 +1695,8 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="24"/>
-      <c r="B54" s="24"/>
+      <c r="A54" s="25"/>
+      <c r="B54" s="25"/>
       <c r="C54" s="1" t="s">
         <v>74</v>
       </c>
@@ -1696,8 +1705,8 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="24"/>
-      <c r="B55" s="24"/>
+      <c r="A55" s="25"/>
+      <c r="B55" s="25"/>
       <c r="C55" s="21" t="s">
         <v>75</v>
       </c>
@@ -1706,8 +1715,8 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="24"/>
-      <c r="B56" s="24"/>
+      <c r="A56" s="25"/>
+      <c r="B56" s="25"/>
       <c r="C56" s="1" t="s">
         <v>76</v>
       </c>
@@ -1716,10 +1725,10 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="24">
+      <c r="A57" s="25">
         <v>17</v>
       </c>
-      <c r="B57" s="24" t="s">
+      <c r="B57" s="25" t="s">
         <v>77</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -1730,8 +1739,8 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="24"/>
-      <c r="B58" s="24"/>
+      <c r="A58" s="25"/>
+      <c r="B58" s="25"/>
       <c r="C58" s="1" t="s">
         <v>79</v>
       </c>
@@ -1740,8 +1749,8 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="24"/>
-      <c r="B59" s="24"/>
+      <c r="A59" s="25"/>
+      <c r="B59" s="25"/>
       <c r="C59" s="1" t="s">
         <v>80</v>
       </c>
@@ -1750,8 +1759,8 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="24"/>
-      <c r="B60" s="24"/>
+      <c r="A60" s="25"/>
+      <c r="B60" s="25"/>
       <c r="C60" s="1" t="s">
         <v>81</v>
       </c>
@@ -1760,10 +1769,10 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="24">
+      <c r="A61" s="25">
         <v>18</v>
       </c>
-      <c r="B61" s="24" t="s">
+      <c r="B61" s="25" t="s">
         <v>82</v>
       </c>
       <c r="C61" s="21" t="s">
@@ -1774,18 +1783,18 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="24"/>
-      <c r="B62" s="24"/>
-      <c r="C62" s="1" t="s">
+      <c r="A62" s="25"/>
+      <c r="B62" s="25"/>
+      <c r="C62" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="D62" s="22" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="24"/>
-      <c r="B63" s="24"/>
+      <c r="A63" s="25"/>
+      <c r="B63" s="25"/>
       <c r="C63" s="1" t="s">
         <v>85</v>
       </c>
@@ -1794,8 +1803,8 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="24"/>
-      <c r="B64" s="24"/>
+      <c r="A64" s="25"/>
+      <c r="B64" s="25"/>
       <c r="C64" s="1" t="s">
         <v>86</v>
       </c>
@@ -1804,10 +1813,10 @@
       </c>
     </row>
     <row r="65" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="24">
+      <c r="A65" s="25">
         <v>19</v>
       </c>
-      <c r="B65" s="24" t="s">
+      <c r="B65" s="25" t="s">
         <v>87</v>
       </c>
       <c r="C65" s="1" t="s">
@@ -1818,8 +1827,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="24"/>
-      <c r="B66" s="24"/>
+      <c r="A66" s="25"/>
+      <c r="B66" s="25"/>
       <c r="C66" s="1" t="s">
         <v>89</v>
       </c>
@@ -1828,8 +1837,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="24"/>
-      <c r="B67" s="24"/>
+      <c r="A67" s="25"/>
+      <c r="B67" s="25"/>
       <c r="C67" s="1" t="s">
         <v>90</v>
       </c>
@@ -1838,8 +1847,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="24"/>
-      <c r="B68" s="24"/>
+      <c r="A68" s="25"/>
+      <c r="B68" s="25"/>
       <c r="C68" s="1" t="s">
         <v>91</v>
       </c>
@@ -1848,10 +1857,10 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="24">
+      <c r="A69" s="25">
         <v>20</v>
       </c>
-      <c r="B69" s="24" t="s">
+      <c r="B69" s="25" t="s">
         <v>92</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -1862,8 +1871,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="24"/>
-      <c r="B70" s="24"/>
+      <c r="A70" s="25"/>
+      <c r="B70" s="25"/>
       <c r="C70" s="1" t="s">
         <v>94</v>
       </c>
@@ -1872,8 +1881,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="24"/>
-      <c r="B71" s="24"/>
+      <c r="A71" s="25"/>
+      <c r="B71" s="25"/>
       <c r="C71" s="1" t="s">
         <v>95</v>
       </c>
@@ -1882,8 +1891,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="24"/>
-      <c r="B72" s="24"/>
+      <c r="A72" s="25"/>
+      <c r="B72" s="25"/>
       <c r="C72" s="1" t="s">
         <v>96</v>
       </c>
@@ -1892,10 +1901,10 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="24">
+      <c r="A73" s="25">
         <v>21</v>
       </c>
-      <c r="B73" s="24" t="s">
+      <c r="B73" s="25" t="s">
         <v>97</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -1906,8 +1915,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
+      <c r="A74" s="25"/>
+      <c r="B74" s="25"/>
       <c r="C74" s="1" t="s">
         <v>99</v>
       </c>
@@ -1916,8 +1925,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
+      <c r="A75" s="25"/>
+      <c r="B75" s="25"/>
       <c r="C75" s="1" t="s">
         <v>100</v>
       </c>
@@ -1926,8 +1935,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
+      <c r="A76" s="25"/>
+      <c r="B76" s="25"/>
       <c r="C76" s="1" t="s">
         <v>101</v>
       </c>
@@ -1936,10 +1945,10 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="24">
+      <c r="A77" s="25">
         <v>22</v>
       </c>
-      <c r="B77" s="24" t="s">
+      <c r="B77" s="25" t="s">
         <v>102</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -1950,8 +1959,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
+      <c r="A78" s="25"/>
+      <c r="B78" s="25"/>
       <c r="C78" s="1" t="s">
         <v>104</v>
       </c>
@@ -1960,8 +1969,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
+      <c r="A79" s="25"/>
+      <c r="B79" s="25"/>
       <c r="C79" s="1" t="s">
         <v>105</v>
       </c>
@@ -1970,8 +1979,8 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
+      <c r="A80" s="25"/>
+      <c r="B80" s="25"/>
       <c r="C80" s="1" t="s">
         <v>106</v>
       </c>
@@ -1980,8 +1989,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
+      <c r="A81" s="25"/>
+      <c r="B81" s="25"/>
       <c r="C81" s="1" t="s">
         <v>107</v>
       </c>
@@ -1990,10 +1999,10 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="24">
+      <c r="A82" s="25">
         <v>23</v>
       </c>
-      <c r="B82" s="24" t="s">
+      <c r="B82" s="25" t="s">
         <v>108</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -2004,8 +2013,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="24"/>
-      <c r="B83" s="24"/>
+      <c r="A83" s="25"/>
+      <c r="B83" s="25"/>
       <c r="C83" s="1" t="s">
         <v>110</v>
       </c>
@@ -2014,8 +2023,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="24"/>
-      <c r="B84" s="24"/>
+      <c r="A84" s="25"/>
+      <c r="B84" s="25"/>
       <c r="C84" s="1" t="s">
         <v>111</v>
       </c>
@@ -2024,10 +2033,10 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="24">
+      <c r="A85" s="25">
         <v>24</v>
       </c>
-      <c r="B85" s="24" t="s">
+      <c r="B85" s="25" t="s">
         <v>112</v>
       </c>
       <c r="C85" s="1" t="s">
@@ -2038,8 +2047,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="24"/>
-      <c r="B86" s="24"/>
+      <c r="A86" s="25"/>
+      <c r="B86" s="25"/>
       <c r="C86" s="1" t="s">
         <v>114</v>
       </c>
@@ -2048,8 +2057,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="24"/>
-      <c r="B87" s="24"/>
+      <c r="A87" s="25"/>
+      <c r="B87" s="25"/>
       <c r="C87" s="1" t="s">
         <v>115</v>
       </c>
@@ -2058,10 +2067,10 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="24">
+      <c r="A88" s="25">
         <v>25</v>
       </c>
-      <c r="B88" s="24" t="s">
+      <c r="B88" s="25" t="s">
         <v>116</v>
       </c>
       <c r="C88" s="1" t="s">
@@ -2072,8 +2081,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="24"/>
-      <c r="B89" s="24"/>
+      <c r="A89" s="25"/>
+      <c r="B89" s="25"/>
       <c r="C89" s="1" t="s">
         <v>118</v>
       </c>
@@ -2082,8 +2091,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="24"/>
-      <c r="B90" s="24"/>
+      <c r="A90" s="25"/>
+      <c r="B90" s="25"/>
       <c r="C90" s="1" t="s">
         <v>119</v>
       </c>
@@ -2092,8 +2101,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="24"/>
-      <c r="B91" s="24"/>
+      <c r="A91" s="25"/>
+      <c r="B91" s="25"/>
       <c r="C91" s="1" t="s">
         <v>120</v>
       </c>

</xml_diff>

<commit_message>
EM-18.3 - Visualização de avaliações dos produtos
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FFF83C-B2CE-4D42-A186-0AE67DD3ADEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63154E7C-855C-44EB-993B-613C46A74184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1785,20 +1785,20 @@
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="25"/>
       <c r="B62" s="25"/>
-      <c r="C62" s="22" t="s">
+      <c r="C62" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="D62" s="22" t="s">
+      <c r="D62" s="21" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="25"/>
       <c r="B63" s="25"/>
-      <c r="C63" s="1" t="s">
+      <c r="C63" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D63" s="22" t="s">
         <v>158</v>
       </c>
     </row>

</xml_diff>